<commit_message>
text function are completed in sheet 2
</commit_message>
<xml_diff>
--- a/CHAPTER6/second.xlsx
+++ b/CHAPTER6/second.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\NITISH_CODE\FOCUSED\SHERYANS_DATASCIENCE\CHAPTER6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBC0CA55-C87A-4EEB-A304-D0DD89CEBED7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FDB87C2-83E6-4D3C-BBF0-A0D82F4FA69A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="6636" xr2:uid="{72805D76-E78E-406D-A531-BADD0BB4DEE4}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="6636" activeTab="2" xr2:uid="{72805D76-E78E-406D-A531-BADD0BB4DEE4}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="FIRST" sheetId="1" r:id="rId1"/>
+    <sheet name="SECOND" sheetId="2" r:id="rId2"/>
+    <sheet name="THIRD" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="79">
   <si>
     <t>Name</t>
   </si>
@@ -106,13 +108,169 @@
   </si>
   <si>
     <t>NESTED IF</t>
+  </si>
+  <si>
+    <t>ERROR HANDLING</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>Aditi</t>
+  </si>
+  <si>
+    <t>North</t>
+  </si>
+  <si>
+    <t>Raj</t>
+  </si>
+  <si>
+    <t>South</t>
+  </si>
+  <si>
+    <t>Meena</t>
+  </si>
+  <si>
+    <t>East</t>
+  </si>
+  <si>
+    <t>Karan</t>
+  </si>
+  <si>
+    <t>West</t>
+  </si>
+  <si>
+    <t>Sonia</t>
+  </si>
+  <si>
+    <t>IFNA</t>
+  </si>
+  <si>
+    <t>IFERROR</t>
+  </si>
+  <si>
+    <t>Full Name</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>aditi.sharma@gmail.com</t>
+  </si>
+  <si>
+    <t>HR-001-IND</t>
+  </si>
+  <si>
+    <t>rajv@outlook.com</t>
+  </si>
+  <si>
+    <t>IT-112-USA</t>
+  </si>
+  <si>
+    <t>meena_k@company.org</t>
+  </si>
+  <si>
+    <t>FIN-345-UK</t>
+  </si>
+  <si>
+    <t>ks@work.net</t>
+  </si>
+  <si>
+    <t>IT-221-AUS</t>
+  </si>
+  <si>
+    <t>SONIA</t>
+  </si>
+  <si>
+    <t>sonia@domain.in</t>
+  </si>
+  <si>
+    <t>HR-019-CAN</t>
+  </si>
+  <si>
+    <t>LEFT</t>
+  </si>
+  <si>
+    <t>RIGHT</t>
+  </si>
+  <si>
+    <t>MID</t>
+  </si>
+  <si>
+    <t>TRIM</t>
+  </si>
+  <si>
+    <t>RAJ     VERMA</t>
+  </si>
+  <si>
+    <t>aditi    sharma</t>
+  </si>
+  <si>
+    <t>karan    singh</t>
+  </si>
+  <si>
+    <t>LENGTH</t>
+  </si>
+  <si>
+    <t>UPPER</t>
+  </si>
+  <si>
+    <t>LOWER</t>
+  </si>
+  <si>
+    <t>PROPER</t>
+  </si>
+  <si>
+    <t>TRIM&amp;PROPER</t>
+  </si>
+  <si>
+    <t>SEARCH</t>
+  </si>
+  <si>
+    <t>FIND</t>
+  </si>
+  <si>
+    <t>USERNAME</t>
+  </si>
+  <si>
+    <t>DEPT</t>
+  </si>
+  <si>
+    <t>SLASH CODE/S</t>
+  </si>
+  <si>
+    <t>SLASH CODE/R</t>
+  </si>
+  <si>
+    <t>CONCAT</t>
+  </si>
+  <si>
+    <t>concat &amp;</t>
+  </si>
+  <si>
+    <t>CCOUNTRY</t>
+  </si>
+  <si>
+    <t>CONTACT</t>
+  </si>
+  <si>
+    <t>TEXT JOIN</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -135,6 +293,40 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -144,7 +336,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -178,11 +370,47 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -191,8 +419,39 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -506,7 +765,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69097A16-DE66-41CC-BBC1-0BDDB17EC869}">
   <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="12.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="4.21875" bestFit="1" customWidth="1"/>
@@ -522,7 +781,7 @@
     <col min="12" max="12" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" ht="15" thickBot="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -560,7 +819,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -607,7 +866,7 @@
         <v>BAD</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -654,7 +913,7 @@
         <v>OK</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
@@ -699,7 +958,7 @@
         <v>GOOD</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
@@ -744,7 +1003,7 @@
         <v>BAD</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12">
       <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
@@ -789,7 +1048,7 @@
         <v>WOW</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12">
       <c r="A7" s="2" t="s">
         <v>14</v>
       </c>
@@ -834,7 +1093,7 @@
         <v>OK</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12">
       <c r="A8" s="2" t="s">
         <v>16</v>
       </c>
@@ -879,7 +1138,7 @@
         <v>BAD</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12">
       <c r="A9" s="2" t="s">
         <v>17</v>
       </c>
@@ -924,7 +1183,7 @@
         <v>GOOD</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12">
       <c r="A10" s="2" t="s">
         <v>18</v>
       </c>
@@ -969,7 +1228,7 @@
         <v>BAD</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -1018,4 +1277,757 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0616A69-200B-4D11-8D35-248E1E34AF47}">
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="33" customHeight="1" thickBot="1">
+      <c r="A1" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+    </row>
+    <row r="2" spans="1:7" ht="16.2" thickBot="1">
+      <c r="A2" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15.6" thickBot="1">
+      <c r="A3" s="4">
+        <v>101</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="4">
+        <v>50000</v>
+      </c>
+      <c r="D3" s="4">
+        <v>55000</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3">
+        <f>_xlfn.IFNA(C3,"NOT AVAILABLE")</f>
+        <v>50000</v>
+      </c>
+      <c r="G3">
+        <f>IFERROR(C3,"ERROR")</f>
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15.6" thickBot="1">
+      <c r="A4" s="4">
+        <v>102</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" s="6" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D4" s="4">
+        <v>60000</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" t="str">
+        <f t="shared" ref="F4:F7" si="0">_xlfn.IFNA(C4,"NOT AVAILABLE")</f>
+        <v>NOT AVAILABLE</v>
+      </c>
+      <c r="G4" t="str">
+        <f t="shared" ref="G4:G7" si="1">IFERROR(C4,"ERROR")</f>
+        <v>ERROR</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15.6" thickBot="1">
+      <c r="A5" s="4">
+        <v>103</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="4">
+        <v>70000</v>
+      </c>
+      <c r="D5" s="4">
+        <v>65000</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="0"/>
+        <v>70000</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="1"/>
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15.6" thickBot="1">
+      <c r="A6" s="4">
+        <v>104</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="6" t="e">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D6" s="4">
+        <v>40000</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F6" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G6" t="str">
+        <f t="shared" si="1"/>
+        <v>ERROR</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.6" thickBot="1">
+      <c r="A7" s="4">
+        <v>105</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="4">
+        <v>45000</v>
+      </c>
+      <c r="D7" s="4">
+        <v>45000</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="0"/>
+        <v>45000</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="1"/>
+        <v>45000</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A802429-D030-4DE5-81FE-6696E2C8C556}">
+  <dimension ref="A1:X6"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" customWidth="1"/>
+    <col min="5" max="7" width="8.88671875" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="11" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="8.88671875" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="25.44140625" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="12.33203125" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="12.5546875" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="17.44140625" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="10" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="8.88671875" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="13.44140625" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="8.88671875" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="15.33203125" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="0" hidden="1" customWidth="1"/>
+    <col min="20" max="21" width="22.21875" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="13.5546875" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="12" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="24.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:24" ht="16.2" thickBot="1">
+      <c r="A1" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="J1" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="K1" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="L1" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="M1" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="N1" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="O1" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="P1" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q1" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="R1" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="S1" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="T1" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="U1" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="V1" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="W1" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="X1" s="10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" ht="16.2" thickBot="1">
+      <c r="A2" s="11">
+        <v>101</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="E2" t="str">
+        <f>LEFT(D2,2)</f>
+        <v>HR</v>
+      </c>
+      <c r="F2" t="str">
+        <f>RIGHT(D2,3)</f>
+        <v>IND</v>
+      </c>
+      <c r="G2" t="str">
+        <f>MID(D2,4,3)</f>
+        <v>001</v>
+      </c>
+      <c r="H2" t="str">
+        <f>TRIM(B2)</f>
+        <v>aditi sharma</v>
+      </c>
+      <c r="I2">
+        <f>LEN(D2)</f>
+        <v>10</v>
+      </c>
+      <c r="J2" t="str">
+        <f>UPPER(C2)</f>
+        <v>ADITI.SHARMA@GMAIL.COM</v>
+      </c>
+      <c r="K2" t="str">
+        <f>LOWER(B2)</f>
+        <v>aditi    sharma</v>
+      </c>
+      <c r="L2" t="str">
+        <f>PROPER(B2)</f>
+        <v>Aditi    Sharma</v>
+      </c>
+      <c r="M2" t="str">
+        <f>PROPER(TRIM(B2))</f>
+        <v>Aditi Sharma</v>
+      </c>
+      <c r="N2">
+        <f>SEARCH("@",C2)</f>
+        <v>13</v>
+      </c>
+      <c r="O2" t="e">
+        <f>FIND("S",B2)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P2" t="str">
+        <f>LEFT(C2,SEARCH("@",C2)-1)</f>
+        <v>aditi.sharma</v>
+      </c>
+      <c r="Q2" t="str">
+        <f>LEFT(D2,SEARCH("-",D2)-1)</f>
+        <v>HR</v>
+      </c>
+      <c r="R2" t="str">
+        <f>SUBSTITUTE(D2,"-","/")</f>
+        <v>HR/001/IND</v>
+      </c>
+      <c r="S2" t="str">
+        <f>REPLACE(D2,3,1,"/")</f>
+        <v>HR/001-IND</v>
+      </c>
+      <c r="T2" t="str">
+        <f>_xlfn.CONCAT(PROPER(TRIM(B2)),"|",D2)</f>
+        <v>Aditi Sharma|HR-001-IND</v>
+      </c>
+      <c r="U2" t="str">
+        <f>PROPER(TRIM(B2))&amp;"|"&amp;D2</f>
+        <v>Aditi Sharma|HR-001-IND</v>
+      </c>
+      <c r="V2" t="str">
+        <f>RIGHT(D2,LEN(D2)-FIND("@",SUBSTITUTE(D2,"-","@",2)))</f>
+        <v>IND</v>
+      </c>
+      <c r="W2">
+        <v>3457345735</v>
+      </c>
+      <c r="X2" t="str">
+        <f>_xlfn.TEXTJOIN(" | ",TRUE,B2,W2)</f>
+        <v>aditi    sharma | 3457345735</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" ht="16.2" thickBot="1">
+      <c r="A3" s="11">
+        <v>102</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E3" t="str">
+        <f t="shared" ref="E3:E6" si="0">LEFT(D3,2)</f>
+        <v>IT</v>
+      </c>
+      <c r="F3" t="str">
+        <f t="shared" ref="F3:F6" si="1">RIGHT(D3,3)</f>
+        <v>USA</v>
+      </c>
+      <c r="G3" t="str">
+        <f t="shared" ref="G3:G6" si="2">MID(D3,4,3)</f>
+        <v>112</v>
+      </c>
+      <c r="H3" t="str">
+        <f t="shared" ref="H3:H6" si="3">TRIM(B3)</f>
+        <v>RAJ VERMA</v>
+      </c>
+      <c r="I3">
+        <f t="shared" ref="I3:I6" si="4">LEN(D3)</f>
+        <v>10</v>
+      </c>
+      <c r="J3" t="str">
+        <f t="shared" ref="J3:J6" si="5">UPPER(C3)</f>
+        <v>RAJV@OUTLOOK.COM</v>
+      </c>
+      <c r="K3" t="str">
+        <f t="shared" ref="K3:K6" si="6">LOWER(B3)</f>
+        <v>raj     verma</v>
+      </c>
+      <c r="L3" t="str">
+        <f t="shared" ref="L3:L6" si="7">PROPER(B3)</f>
+        <v>Raj     Verma</v>
+      </c>
+      <c r="M3" t="str">
+        <f t="shared" ref="M3:M6" si="8">PROPER(TRIM(B3))</f>
+        <v>Raj Verma</v>
+      </c>
+      <c r="N3">
+        <f t="shared" ref="N3:N6" si="9">SEARCH("@",C3)</f>
+        <v>5</v>
+      </c>
+      <c r="O3" t="e">
+        <f t="shared" ref="O3:O6" si="10">FIND("S",B3)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P3" t="str">
+        <f t="shared" ref="P3:P6" si="11">LEFT(C3,SEARCH("@",C3)-1)</f>
+        <v>rajv</v>
+      </c>
+      <c r="Q3" t="str">
+        <f t="shared" ref="Q3:Q6" si="12">LEFT(D3,SEARCH("-",D3)-1)</f>
+        <v>IT</v>
+      </c>
+      <c r="R3" t="str">
+        <f t="shared" ref="R3:R6" si="13">SUBSTITUTE(D3,"-","/")</f>
+        <v>IT/112/USA</v>
+      </c>
+      <c r="S3" t="str">
+        <f t="shared" ref="S3:S6" si="14">REPLACE(D3,3,1,"/")</f>
+        <v>IT/112-USA</v>
+      </c>
+      <c r="T3" t="str">
+        <f t="shared" ref="T3:T6" si="15">_xlfn.CONCAT(PROPER(TRIM(B3)),"|",D3)</f>
+        <v>Raj Verma|IT-112-USA</v>
+      </c>
+      <c r="U3" t="str">
+        <f t="shared" ref="U3:U6" si="16">PROPER(TRIM(B3))&amp;"|"&amp;D3</f>
+        <v>Raj Verma|IT-112-USA</v>
+      </c>
+      <c r="V3" t="str">
+        <f t="shared" ref="V3:V6" si="17">RIGHT(D3,LEN(D3)-FIND("@",SUBSTITUTE(D3,"-","@",2)))</f>
+        <v>USA</v>
+      </c>
+      <c r="X3" t="str">
+        <f t="shared" ref="X3:X6" si="18">_xlfn.TEXTJOIN(" | ",TRUE,B3,W3)</f>
+        <v>RAJ     VERMA</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" ht="16.2" thickBot="1">
+      <c r="A4" s="11">
+        <v>103</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="E4" t="str">
+        <f t="shared" si="0"/>
+        <v>FI</v>
+      </c>
+      <c r="F4" t="str">
+        <f t="shared" si="1"/>
+        <v>-UK</v>
+      </c>
+      <c r="G4" t="str">
+        <f t="shared" si="2"/>
+        <v>-34</v>
+      </c>
+      <c r="H4" t="str">
+        <f t="shared" si="3"/>
+        <v>Meena</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="4"/>
+        <v>10</v>
+      </c>
+      <c r="J4" t="str">
+        <f t="shared" si="5"/>
+        <v>MEENA_K@COMPANY.ORG</v>
+      </c>
+      <c r="K4" t="str">
+        <f t="shared" si="6"/>
+        <v>meena</v>
+      </c>
+      <c r="L4" t="str">
+        <f t="shared" si="7"/>
+        <v>Meena</v>
+      </c>
+      <c r="M4" t="str">
+        <f t="shared" si="8"/>
+        <v>Meena</v>
+      </c>
+      <c r="N4">
+        <f t="shared" si="9"/>
+        <v>8</v>
+      </c>
+      <c r="O4" t="e">
+        <f t="shared" si="10"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P4" t="str">
+        <f t="shared" si="11"/>
+        <v>meena_k</v>
+      </c>
+      <c r="Q4" t="str">
+        <f t="shared" si="12"/>
+        <v>FIN</v>
+      </c>
+      <c r="R4" t="str">
+        <f t="shared" si="13"/>
+        <v>FIN/345/UK</v>
+      </c>
+      <c r="S4" t="str">
+        <f t="shared" si="14"/>
+        <v>FI/-345-UK</v>
+      </c>
+      <c r="T4" t="str">
+        <f t="shared" si="15"/>
+        <v>Meena|FIN-345-UK</v>
+      </c>
+      <c r="U4" t="str">
+        <f t="shared" si="16"/>
+        <v>Meena|FIN-345-UK</v>
+      </c>
+      <c r="V4" t="str">
+        <f t="shared" si="17"/>
+        <v>UK</v>
+      </c>
+      <c r="W4">
+        <v>3457345573</v>
+      </c>
+      <c r="X4" t="str">
+        <f t="shared" si="18"/>
+        <v>Meena | 3457345573</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" ht="16.2" thickBot="1">
+      <c r="A5" s="11">
+        <v>104</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="E5" t="str">
+        <f t="shared" si="0"/>
+        <v>IT</v>
+      </c>
+      <c r="F5" t="str">
+        <f t="shared" si="1"/>
+        <v>AUS</v>
+      </c>
+      <c r="G5" t="str">
+        <f t="shared" si="2"/>
+        <v>221</v>
+      </c>
+      <c r="H5" t="str">
+        <f t="shared" si="3"/>
+        <v>karan singh</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="4"/>
+        <v>10</v>
+      </c>
+      <c r="J5" t="str">
+        <f t="shared" si="5"/>
+        <v>KS@WORK.NET</v>
+      </c>
+      <c r="K5" t="str">
+        <f t="shared" si="6"/>
+        <v>karan    singh</v>
+      </c>
+      <c r="L5" t="str">
+        <f t="shared" si="7"/>
+        <v>Karan    Singh</v>
+      </c>
+      <c r="M5" t="str">
+        <f t="shared" si="8"/>
+        <v>Karan Singh</v>
+      </c>
+      <c r="N5">
+        <f t="shared" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="O5" t="e">
+        <f t="shared" si="10"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P5" t="str">
+        <f t="shared" si="11"/>
+        <v>ks</v>
+      </c>
+      <c r="Q5" t="str">
+        <f t="shared" si="12"/>
+        <v>IT</v>
+      </c>
+      <c r="R5" t="str">
+        <f t="shared" si="13"/>
+        <v>IT/221/AUS</v>
+      </c>
+      <c r="S5" t="str">
+        <f t="shared" si="14"/>
+        <v>IT/221-AUS</v>
+      </c>
+      <c r="T5" t="str">
+        <f t="shared" si="15"/>
+        <v>Karan Singh|IT-221-AUS</v>
+      </c>
+      <c r="U5" t="str">
+        <f t="shared" si="16"/>
+        <v>Karan Singh|IT-221-AUS</v>
+      </c>
+      <c r="V5" t="str">
+        <f t="shared" si="17"/>
+        <v>AUS</v>
+      </c>
+      <c r="X5" t="str">
+        <f t="shared" si="18"/>
+        <v>karan    singh</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" ht="16.2" thickBot="1">
+      <c r="A6" s="11">
+        <v>105</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="E6" t="str">
+        <f t="shared" si="0"/>
+        <v>HR</v>
+      </c>
+      <c r="F6" t="str">
+        <f t="shared" si="1"/>
+        <v>CAN</v>
+      </c>
+      <c r="G6" t="str">
+        <f t="shared" si="2"/>
+        <v>019</v>
+      </c>
+      <c r="H6" t="str">
+        <f t="shared" si="3"/>
+        <v>SONIA</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="4"/>
+        <v>10</v>
+      </c>
+      <c r="J6" t="str">
+        <f t="shared" si="5"/>
+        <v>SONIA@DOMAIN.IN</v>
+      </c>
+      <c r="K6" t="str">
+        <f t="shared" si="6"/>
+        <v>sonia</v>
+      </c>
+      <c r="L6" t="str">
+        <f t="shared" si="7"/>
+        <v>Sonia</v>
+      </c>
+      <c r="M6" t="str">
+        <f t="shared" si="8"/>
+        <v>Sonia</v>
+      </c>
+      <c r="N6">
+        <f t="shared" si="9"/>
+        <v>6</v>
+      </c>
+      <c r="O6">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="P6" t="str">
+        <f t="shared" si="11"/>
+        <v>sonia</v>
+      </c>
+      <c r="Q6" t="str">
+        <f t="shared" si="12"/>
+        <v>HR</v>
+      </c>
+      <c r="R6" t="str">
+        <f t="shared" si="13"/>
+        <v>HR/019/CAN</v>
+      </c>
+      <c r="S6" t="str">
+        <f t="shared" si="14"/>
+        <v>HR/019-CAN</v>
+      </c>
+      <c r="T6" t="str">
+        <f t="shared" si="15"/>
+        <v>Sonia|HR-019-CAN</v>
+      </c>
+      <c r="U6" t="str">
+        <f t="shared" si="16"/>
+        <v>Sonia|HR-019-CAN</v>
+      </c>
+      <c r="V6" t="str">
+        <f t="shared" si="17"/>
+        <v>CAN</v>
+      </c>
+      <c r="W6">
+        <v>7245734573</v>
+      </c>
+      <c r="X6" t="str">
+        <f t="shared" si="18"/>
+        <v>SONIA | 7245734573</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" display="mailto:aditi.sharma@gmail.com" xr:uid="{D9667B33-690E-4A3C-9388-E44F4B47A147}"/>
+    <hyperlink ref="C3" r:id="rId2" display="mailto:rajv@outlook.com" xr:uid="{7E385210-64B2-4E05-AD75-B997B9797200}"/>
+    <hyperlink ref="C4" r:id="rId3" display="mailto:meena_k@company.org" xr:uid="{21DD55CC-A288-440C-81DF-ED7042CC95FE}"/>
+    <hyperlink ref="C5" r:id="rId4" display="mailto:ks@work.net" xr:uid="{34E21C9A-3312-4730-9DCC-D9AD3CCB68D0}"/>
+    <hyperlink ref="C6" r:id="rId5" display="mailto:sonia@domain.in" xr:uid="{B885EFFC-928C-4053-8993-6C3E052F956F}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
date time is completed
</commit_message>
<xml_diff>
--- a/CHAPTER6/second.xlsx
+++ b/CHAPTER6/second.xlsx
@@ -8,14 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\NITISH_CODE\FOCUSED\SHERYANS_DATASCIENCE\CHAPTER6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FDB87C2-83E6-4D3C-BBF0-A0D82F4FA69A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13245AAA-5C42-4F77-BB09-54CA304BF510}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="6636" activeTab="2" xr2:uid="{72805D76-E78E-406D-A531-BADD0BB4DEE4}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="6636" firstSheet="1" activeTab="4" xr2:uid="{72805D76-E78E-406D-A531-BADD0BB4DEE4}"/>
   </bookViews>
   <sheets>
     <sheet name="FIRST" sheetId="1" r:id="rId1"/>
     <sheet name="SECOND" sheetId="2" r:id="rId2"/>
     <sheet name="THIRD" sheetId="3" r:id="rId3"/>
+    <sheet name="FOURTH" sheetId="4" r:id="rId4"/>
+    <sheet name="FIFTH" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="96">
   <si>
     <t>Name</t>
   </si>
@@ -264,13 +266,64 @@
   </si>
   <si>
     <t>TEXT JOIN</t>
+  </si>
+  <si>
+    <t>DATE AND TIME</t>
+  </si>
+  <si>
+    <t>Join Date</t>
+  </si>
+  <si>
+    <t>End Date</t>
+  </si>
+  <si>
+    <t>DOB</t>
+  </si>
+  <si>
+    <t>DAY</t>
+  </si>
+  <si>
+    <t>MONTH</t>
+  </si>
+  <si>
+    <t>YEAR</t>
+  </si>
+  <si>
+    <t>WEEKNUM</t>
+  </si>
+  <si>
+    <t>DATE DIF</t>
+  </si>
+  <si>
+    <t>WORKING DAYS</t>
+  </si>
+  <si>
+    <t>EOMONTH</t>
+  </si>
+  <si>
+    <t>EmpID</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Delhi</t>
+  </si>
+  <si>
+    <t>Mumbai</t>
+  </si>
+  <si>
+    <t>Bangalore</t>
+  </si>
+  <si>
+    <t>Pune</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -323,6 +376,14 @@
       <u/>
       <sz val="12"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -410,7 +471,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -428,12 +489,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -448,6 +503,26 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1294,34 +1369,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="33" customHeight="1" thickBot="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
     </row>
     <row r="2" spans="1:7" ht="16.2" thickBot="1">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="8" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1468,110 +1543,110 @@
     <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.77734375" customWidth="1"/>
-    <col min="5" max="7" width="8.88671875" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="11" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="8.88671875" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="25.44140625" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="12.33203125" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="12.5546875" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="17.44140625" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="10" hidden="1" customWidth="1"/>
-    <col min="15" max="15" width="8.88671875" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="13.44140625" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="8.88671875" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="15.33203125" hidden="1" customWidth="1"/>
-    <col min="19" max="19" width="0" hidden="1" customWidth="1"/>
-    <col min="20" max="21" width="22.21875" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="13.5546875" hidden="1" customWidth="1"/>
+    <col min="5" max="7" width="8.88671875" customWidth="1"/>
+    <col min="8" max="8" width="11" customWidth="1"/>
+    <col min="9" max="9" width="8.88671875" customWidth="1"/>
+    <col min="10" max="10" width="25.44140625" customWidth="1"/>
+    <col min="11" max="11" width="12.33203125" customWidth="1"/>
+    <col min="12" max="12" width="12.5546875" customWidth="1"/>
+    <col min="13" max="13" width="17.44140625" customWidth="1"/>
+    <col min="14" max="14" width="10" customWidth="1"/>
+    <col min="15" max="15" width="8.88671875" customWidth="1"/>
+    <col min="16" max="16" width="13.44140625" customWidth="1"/>
+    <col min="17" max="17" width="8.88671875" customWidth="1"/>
+    <col min="18" max="18" width="15.33203125" customWidth="1"/>
+    <col min="19" max="19" width="8.88671875" customWidth="1"/>
+    <col min="20" max="21" width="22.21875" customWidth="1"/>
+    <col min="22" max="22" width="13.5546875" customWidth="1"/>
     <col min="23" max="23" width="12" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="24.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="16.2" thickBot="1">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="I1" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="J1" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="K1" s="10" t="s">
+      <c r="K1" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="L1" s="10" t="s">
+      <c r="L1" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="M1" s="10" t="s">
+      <c r="M1" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="N1" s="10" t="s">
+      <c r="N1" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="O1" s="10" t="s">
+      <c r="O1" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="P1" s="10" t="s">
+      <c r="P1" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="Q1" s="10" t="s">
+      <c r="Q1" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="R1" s="10" t="s">
+      <c r="R1" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="S1" s="10" t="s">
+      <c r="S1" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="T1" s="10" t="s">
+      <c r="T1" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="U1" s="10" t="s">
+      <c r="U1" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="V1" s="10" t="s">
+      <c r="V1" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="W1" s="10" t="s">
+      <c r="W1" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="X1" s="10" t="s">
+      <c r="X1" s="8" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:24" ht="16.2" thickBot="1">
-      <c r="A2" s="11">
+      <c r="A2" s="9">
         <v>101</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="10" t="s">
         <v>46</v>
       </c>
       <c r="E2" t="str">
@@ -1655,16 +1730,16 @@
       </c>
     </row>
     <row r="3" spans="1:24" ht="16.2" thickBot="1">
-      <c r="A3" s="11">
+      <c r="A3" s="9">
         <v>102</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="10" t="s">
         <v>48</v>
       </c>
       <c r="E3" t="str">
@@ -1745,16 +1820,16 @@
       </c>
     </row>
     <row r="4" spans="1:24" ht="16.2" thickBot="1">
-      <c r="A4" s="11">
+      <c r="A4" s="9">
         <v>103</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="10" t="s">
         <v>50</v>
       </c>
       <c r="E4" t="str">
@@ -1838,16 +1913,16 @@
       </c>
     </row>
     <row r="5" spans="1:24" ht="16.2" thickBot="1">
-      <c r="A5" s="11">
+      <c r="A5" s="9">
         <v>104</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="10" t="s">
         <v>52</v>
       </c>
       <c r="E5" t="str">
@@ -1928,16 +2003,16 @@
       </c>
     </row>
     <row r="6" spans="1:24" ht="16.2" thickBot="1">
-      <c r="A6" s="11">
+      <c r="A6" s="9">
         <v>105</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="10" t="s">
         <v>55</v>
       </c>
       <c r="E6" t="str">
@@ -2030,4 +2105,434 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C69FE283-BA4B-47E0-94BB-B5C6B58FB6FB}">
+  <dimension ref="A1:L13"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.44140625" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="9.21875" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="6.88671875" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5546875" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="11" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="18.6640625" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="12.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="24" thickBot="1">
+      <c r="A1" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+    </row>
+    <row r="2" spans="1:12" ht="16.2" thickBot="1">
+      <c r="A2" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="L2" s="8" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="15.6" thickBot="1">
+      <c r="A3" s="4">
+        <v>101</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="15">
+        <v>44562</v>
+      </c>
+      <c r="D3" s="15">
+        <v>45657</v>
+      </c>
+      <c r="E3" s="15">
+        <v>36022</v>
+      </c>
+      <c r="F3">
+        <f>DAY(C3)</f>
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <f>MONTH(C3)</f>
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <f>YEAR(C3)</f>
+        <v>2022</v>
+      </c>
+      <c r="I3">
+        <f>WEEKNUM(C3,2)</f>
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <f ca="1">DATEDIF(C3,TODAY(),"D")</f>
+        <v>1750</v>
+      </c>
+      <c r="K3">
+        <f>NETWORKDAYS(C3,D3)</f>
+        <v>782</v>
+      </c>
+      <c r="L3" s="17">
+        <f>EOMONTH(C3,-2)</f>
+        <v>44530</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="15.6" thickBot="1">
+      <c r="A4" s="4">
+        <v>102</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" s="15">
+        <v>44270</v>
+      </c>
+      <c r="D4" s="15">
+        <v>45731</v>
+      </c>
+      <c r="E4" s="15">
+        <v>33166</v>
+      </c>
+      <c r="F4">
+        <f t="shared" ref="F4:F7" si="0">DAY(C4)</f>
+        <v>15</v>
+      </c>
+      <c r="G4">
+        <f t="shared" ref="G4:G7" si="1">MONTH(C4)</f>
+        <v>3</v>
+      </c>
+      <c r="H4">
+        <f t="shared" ref="H4:H7" si="2">YEAR(C4)</f>
+        <v>2021</v>
+      </c>
+      <c r="I4">
+        <f t="shared" ref="I4:I7" si="3">WEEKNUM(C4)</f>
+        <v>12</v>
+      </c>
+      <c r="J4">
+        <f t="shared" ref="J4:J7" ca="1" si="4">DATEDIF(C4,TODAY(),"D")</f>
+        <v>2042</v>
+      </c>
+      <c r="K4">
+        <f t="shared" ref="K4:K7" si="5">NETWORKDAYS(C4,D4)</f>
+        <v>1045</v>
+      </c>
+      <c r="L4" s="17">
+        <f t="shared" ref="L4:L7" si="6">EOMONTH(C4,-2)</f>
+        <v>44227</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="15.6" thickBot="1">
+      <c r="A5" s="4">
+        <v>103</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="15">
+        <v>44022</v>
+      </c>
+      <c r="D5" s="15">
+        <v>45116</v>
+      </c>
+      <c r="E5" s="15">
+        <v>34704</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="H5">
+        <f t="shared" si="2"/>
+        <v>2020</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="3"/>
+        <v>28</v>
+      </c>
+      <c r="J5">
+        <f t="shared" ca="1" si="4"/>
+        <v>2290</v>
+      </c>
+      <c r="K5">
+        <f t="shared" si="5"/>
+        <v>781</v>
+      </c>
+      <c r="L5" s="17">
+        <f t="shared" si="6"/>
+        <v>43982</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="15.6" thickBot="1">
+      <c r="A6" s="4">
+        <v>104</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="15">
+        <v>44958</v>
+      </c>
+      <c r="D6" s="15">
+        <v>46053</v>
+      </c>
+      <c r="E6" s="15">
+        <v>32478</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="H6">
+        <f t="shared" si="2"/>
+        <v>2023</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="J6">
+        <f t="shared" ca="1" si="4"/>
+        <v>1354</v>
+      </c>
+      <c r="K6">
+        <f t="shared" si="5"/>
+        <v>783</v>
+      </c>
+      <c r="L6" s="17">
+        <f t="shared" si="6"/>
+        <v>44926</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="15.6" thickBot="1">
+      <c r="A7" s="4">
+        <v>105</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="15">
+        <v>44920</v>
+      </c>
+      <c r="D7" s="15">
+        <v>45651</v>
+      </c>
+      <c r="E7" s="15">
+        <v>33734</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="1"/>
+        <v>12</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="2"/>
+        <v>2022</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="3"/>
+        <v>53</v>
+      </c>
+      <c r="J7">
+        <f t="shared" ca="1" si="4"/>
+        <v>1392</v>
+      </c>
+      <c r="K7">
+        <f t="shared" si="5"/>
+        <v>523</v>
+      </c>
+      <c r="L7" s="17">
+        <f t="shared" si="6"/>
+        <v>44865</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="C12" s="17">
+        <f ca="1">TODAY()</f>
+        <v>46312</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="C13" s="18">
+        <f ca="1">NOW()</f>
+        <v>46312.452766898146</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83B39815-1302-4725-9013-3D3086431F15}">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="16.2" thickBot="1">
+      <c r="A1" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15.6" thickBot="1">
+      <c r="A2" s="9">
+        <v>101</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="19">
+        <v>40000</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15.6" thickBot="1">
+      <c r="A3" s="9">
+        <v>102</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="19">
+        <v>65000</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15.6" thickBot="1">
+      <c r="A4" s="9">
+        <v>103</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="19">
+        <v>55000</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15.6" thickBot="1">
+      <c r="A5" s="9">
+        <v>104</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="19">
+        <v>80000</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15.6" thickBot="1">
+      <c r="A6" s="9">
+        <v>105</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="19">
+        <v>50000</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>